<commit_message>
Update Philly BYOB Restaurant_with_latlng.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/geocode_full/Philly BYOB Restaurant_with_latlng.xlsx
+++ b/philly_yelp_crawler/data/geocode_full/Philly BYOB Restaurant_with_latlng.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\geocode_full\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF262DCB-2114-4674-9F77-1D8C0E710EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC5176E-248B-473C-97BF-5CC21204BEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="153">
   <si>
     <t>Name</t>
   </si>
@@ -236,15 +236,6 @@
   </si>
   <si>
     <t>214 South St, Philadelphia, PA 19147, United States</t>
-  </si>
-  <si>
-    <t>La Sera Italiana BYOB</t>
-  </si>
-  <si>
-    <t>1608 South St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
-    <t>(267) 930-7805</t>
   </si>
   <si>
     <t>La Viola Bistro</t>
@@ -859,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.875" customWidth="1"/>
@@ -1330,10 +1321,10 @@
         <v>74</v>
       </c>
       <c r="D21">
-        <v>39.943967499999999</v>
+        <v>39.947770800000001</v>
       </c>
       <c r="E21">
-        <v>-75.169153299999991</v>
+        <v>-75.167849599999997</v>
       </c>
       <c r="F21" t="s">
         <v>10</v>
@@ -1353,10 +1344,10 @@
         <v>77</v>
       </c>
       <c r="D22">
-        <v>39.947770800000001</v>
+        <v>39.9196271</v>
       </c>
       <c r="E22">
-        <v>-75.167849599999997</v>
+        <v>-75.171403699999999</v>
       </c>
       <c r="F22" t="s">
         <v>10</v>
@@ -1376,10 +1367,10 @@
         <v>80</v>
       </c>
       <c r="D23">
-        <v>39.9196271</v>
+        <v>39.939456999999997</v>
       </c>
       <c r="E23">
-        <v>-75.171403699999999</v>
+        <v>-75.171263500000009</v>
       </c>
       <c r="F23" t="s">
         <v>10</v>
@@ -1399,39 +1390,39 @@
         <v>83</v>
       </c>
       <c r="D24">
-        <v>39.939456999999997</v>
+        <v>39.940005499999998</v>
       </c>
       <c r="E24">
-        <v>-75.171263500000009</v>
+        <v>-75.152943699999994</v>
       </c>
       <c r="F24" t="s">
         <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
+        <v>87</v>
+      </c>
+      <c r="D25">
+        <v>39.9496781</v>
+      </c>
+      <c r="E25">
+        <v>-75.1738043</v>
+      </c>
+      <c r="F25" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" t="s">
         <v>86</v>
-      </c>
-      <c r="D25">
-        <v>39.940005499999998</v>
-      </c>
-      <c r="E25">
-        <v>-75.152943699999994</v>
-      </c>
-      <c r="F25" t="s">
-        <v>10</v>
-      </c>
-      <c r="G25" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1441,20 +1432,17 @@
       <c r="B26" t="s">
         <v>89</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26">
+        <v>39.939949299999988</v>
+      </c>
+      <c r="E26">
+        <v>-75.157774399999994</v>
+      </c>
+      <c r="F26" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" t="s">
         <v>90</v>
-      </c>
-      <c r="D26">
-        <v>39.9496781</v>
-      </c>
-      <c r="E26">
-        <v>-75.1738043</v>
-      </c>
-      <c r="F26" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1464,17 +1452,20 @@
       <c r="B27" t="s">
         <v>92</v>
       </c>
+      <c r="C27" t="s">
+        <v>93</v>
+      </c>
       <c r="D27">
-        <v>39.939949299999988</v>
+        <v>39.951250900000012</v>
       </c>
       <c r="E27">
-        <v>-75.157774399999994</v>
+        <v>-75.174123500000007</v>
       </c>
       <c r="F27" t="s">
         <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1488,10 +1479,10 @@
         <v>96</v>
       </c>
       <c r="D28">
-        <v>39.951250900000012</v>
+        <v>39.946510799999999</v>
       </c>
       <c r="E28">
-        <v>-75.174123500000007</v>
+        <v>-75.1617818</v>
       </c>
       <c r="F28" t="s">
         <v>10</v>
@@ -1511,39 +1502,39 @@
         <v>99</v>
       </c>
       <c r="D29">
-        <v>39.946510799999999</v>
+        <v>39.953597799999997</v>
       </c>
       <c r="E29">
-        <v>-75.1617818</v>
+        <v>-75.160984799999994</v>
       </c>
       <c r="F29" t="s">
         <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B30" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C30" t="s">
+        <v>103</v>
+      </c>
+      <c r="D30">
+        <v>39.944041200000001</v>
+      </c>
+      <c r="E30">
+        <v>-75.170019699999997</v>
+      </c>
+      <c r="F30" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" t="s">
         <v>102</v>
-      </c>
-      <c r="D30">
-        <v>39.953597799999997</v>
-      </c>
-      <c r="E30">
-        <v>-75.160984799999994</v>
-      </c>
-      <c r="F30" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
@@ -1557,131 +1548,131 @@
         <v>106</v>
       </c>
       <c r="D31">
-        <v>39.944041200000001</v>
+        <v>39.951966800000001</v>
       </c>
       <c r="E31">
-        <v>-75.170019699999997</v>
+        <v>-75.144375400000015</v>
       </c>
       <c r="F31" t="s">
         <v>10</v>
       </c>
       <c r="G31" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D32">
-        <v>39.951966800000001</v>
+        <v>39.936847999999998</v>
       </c>
       <c r="E32">
-        <v>-75.144375400000015</v>
+        <v>-75.156487599999991</v>
       </c>
       <c r="F32" t="s">
         <v>10</v>
       </c>
       <c r="G32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D33">
-        <v>39.936847999999998</v>
+        <v>39.965312599999997</v>
       </c>
       <c r="E33">
-        <v>-75.156487599999991</v>
+        <v>-75.140657599999997</v>
       </c>
       <c r="F33" t="s">
         <v>10</v>
       </c>
       <c r="G33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B34" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C34" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D34">
-        <v>39.965312599999997</v>
+        <v>39.951410799999998</v>
       </c>
       <c r="E34">
-        <v>-75.140657599999997</v>
+        <v>-75.17510399999999</v>
       </c>
       <c r="F34" t="s">
         <v>10</v>
       </c>
       <c r="G34" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D35">
-        <v>39.951410799999998</v>
+        <v>39.926310399999998</v>
       </c>
       <c r="E35">
-        <v>-75.17510399999999</v>
+        <v>-75.167529000000002</v>
       </c>
       <c r="F35" t="s">
         <v>10</v>
       </c>
       <c r="G35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B36" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C36" t="s">
+        <v>126</v>
+      </c>
+      <c r="D36">
+        <v>39.943962999999997</v>
+      </c>
+      <c r="E36">
+        <v>-75.167322100000007</v>
+      </c>
+      <c r="F36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" t="s">
         <v>125</v>
-      </c>
-      <c r="D36">
-        <v>39.926310399999998</v>
-      </c>
-      <c r="E36">
-        <v>-75.167529000000002</v>
-      </c>
-      <c r="F36" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
@@ -1695,85 +1686,85 @@
         <v>129</v>
       </c>
       <c r="D37">
-        <v>39.943962999999997</v>
+        <v>39.919344299999999</v>
       </c>
       <c r="E37">
-        <v>-75.167322100000007</v>
+        <v>-75.171028399999997</v>
       </c>
       <c r="F37" t="s">
         <v>10</v>
       </c>
       <c r="G37" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D38">
-        <v>39.919344299999999</v>
+        <v>39.925141500000002</v>
       </c>
       <c r="E38">
-        <v>-75.171028399999997</v>
+        <v>-75.174745099999996</v>
       </c>
       <c r="F38" t="s">
         <v>10</v>
       </c>
       <c r="G38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D39">
-        <v>39.925141500000002</v>
+        <v>39.933937399999998</v>
       </c>
       <c r="E39">
-        <v>-75.174745099999996</v>
+        <v>-75.155578599999998</v>
       </c>
       <c r="F39" t="s">
         <v>10</v>
       </c>
       <c r="G39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B40" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C40" t="s">
+        <v>141</v>
+      </c>
+      <c r="D40">
+        <v>39.942575300000001</v>
+      </c>
+      <c r="E40">
+        <v>-75.1853081</v>
+      </c>
+      <c r="F40" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40" t="s">
         <v>140</v>
-      </c>
-      <c r="D40">
-        <v>39.933937399999998</v>
-      </c>
-      <c r="E40">
-        <v>-75.155578599999998</v>
-      </c>
-      <c r="F40" t="s">
-        <v>10</v>
-      </c>
-      <c r="G40" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
@@ -1787,10 +1778,10 @@
         <v>144</v>
       </c>
       <c r="D41">
-        <v>39.942575300000001</v>
+        <v>39.948727300000002</v>
       </c>
       <c r="E41">
-        <v>-75.1853081</v>
+        <v>-75.177952800000014</v>
       </c>
       <c r="F41" t="s">
         <v>10</v>
@@ -1810,62 +1801,39 @@
         <v>147</v>
       </c>
       <c r="D42">
-        <v>39.948727300000002</v>
+        <v>39.951509600000001</v>
       </c>
       <c r="E42">
-        <v>-75.177952800000014</v>
+        <v>-75.1748482</v>
       </c>
       <c r="F42" t="s">
         <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B43" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C43" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D43">
-        <v>39.951509600000001</v>
+        <v>39.948377800000003</v>
       </c>
       <c r="E43">
-        <v>-75.1748482</v>
+        <v>-75.217939799999996</v>
       </c>
       <c r="F43" t="s">
         <v>10</v>
       </c>
       <c r="G43" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
         <v>152</v>
-      </c>
-      <c r="B44" t="s">
-        <v>153</v>
-      </c>
-      <c r="C44" t="s">
-        <v>154</v>
-      </c>
-      <c r="D44">
-        <v>39.948377800000003</v>
-      </c>
-      <c r="E44">
-        <v>-75.217939799999996</v>
-      </c>
-      <c r="F44" t="s">
-        <v>10</v>
-      </c>
-      <c r="G44" t="s">
-        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>